<commit_message>
feat: implement DashboardController for audit metrics and add export template file
</commit_message>
<xml_diff>
--- a/public/tamplate-xlsx/Internal_Audit_Export_Tamplate.xlsx
+++ b/public/tamplate-xlsx/Internal_Audit_Export_Tamplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ICT\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ict\www-wsl\qms\public\tamplate-xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1B735F-3FF6-4730-9D6D-A11EB43868A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EFB13E8-5AC0-401D-98A7-6587E5BE66AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -82,13 +82,7 @@
     <t>CAR NO</t>
   </si>
   <si>
-    <t>CLAUSE NO</t>
-  </si>
-  <si>
     <t>Audit Category</t>
-  </si>
-  <si>
-    <t>Part No/Name</t>
   </si>
   <si>
     <t>Dept</t>
@@ -174,6 +168,12 @@
     <t>1. Preventive Action 1
 2. Preventive Action 2
 3. Preventive Action 3</t>
+  </si>
+  <si>
+    <t>CLAUSE TITLE</t>
+  </si>
+  <si>
+    <t>Part No/Part Name/Process Checked</t>
   </si>
 </sst>
 </file>
@@ -438,16 +438,7 @@
     <xf numFmtId="15" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -462,21 +453,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -492,7 +474,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -961,8 +961,11 @@
     <col min="2" max="2" width="5.42578125" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
     <col min="10" max="11" width="12.5703125" customWidth="1"/>
-    <col min="13" max="13" width="39.28515625" customWidth="1"/>
+    <col min="13" max="13" width="36.5703125" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" customWidth="1"/>
     <col min="16" max="16" width="28.85546875" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" customWidth="1"/>
     <col min="18" max="18" width="28.85546875" customWidth="1"/>
@@ -973,105 +976,105 @@
       <c r="B2" s="1"/>
       <c r="C2" s="2"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="27"/>
-      <c r="P2" s="27"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27"/>
-      <c r="S2" s="32"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="25"/>
     </row>
     <row r="3" spans="2:19" ht="15" customHeight="1">
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33"/>
-      <c r="Q3" s="33"/>
-      <c r="R3" s="33"/>
-      <c r="S3" s="34"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="27"/>
+      <c r="N3" s="27"/>
+      <c r="O3" s="27"/>
+      <c r="P3" s="27"/>
+      <c r="Q3" s="27"/>
+      <c r="R3" s="27"/>
+      <c r="S3" s="28"/>
     </row>
     <row r="4" spans="2:19" ht="15.75" customHeight="1">
       <c r="B4" s="4"/>
       <c r="C4" s="7"/>
       <c r="D4" s="8"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
-      <c r="Q4" s="33"/>
-      <c r="R4" s="33"/>
-      <c r="S4" s="34"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="27"/>
+      <c r="S4" s="28"/>
     </row>
     <row r="5" spans="2:19" ht="15.75" customHeight="1">
       <c r="B5" s="4"/>
       <c r="C5" s="7"/>
       <c r="D5" s="8"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
-      <c r="K5" s="33"/>
-      <c r="L5" s="33"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="33"/>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="33"/>
-      <c r="R5" s="33"/>
-      <c r="S5" s="34"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="27"/>
+      <c r="S5" s="28"/>
     </row>
     <row r="6" spans="2:19" ht="15" customHeight="1">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36"/>
-      <c r="L6" s="36"/>
-      <c r="M6" s="36"/>
-      <c r="N6" s="36"/>
-      <c r="O6" s="36"/>
-      <c r="P6" s="36"/>
-      <c r="Q6" s="36"/>
-      <c r="R6" s="36"/>
-      <c r="S6" s="37"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="30"/>
+      <c r="N6" s="30"/>
+      <c r="O6" s="30"/>
+      <c r="P6" s="30"/>
+      <c r="Q6" s="30"/>
+      <c r="R6" s="30"/>
+      <c r="S6" s="31"/>
     </row>
     <row r="7" spans="2:19">
       <c r="B7" s="9"/>
@@ -1124,80 +1127,80 @@
       </c>
     </row>
     <row r="8" spans="2:19">
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="G8" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="I8" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="J8" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="I8" s="24" t="s">
+      <c r="K8" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="J8" s="24" t="s">
+      <c r="L8" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="K8" s="24" t="s">
+      <c r="M8" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="24" t="s">
+      <c r="N8" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="M8" s="24" t="s">
+      <c r="O8" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="N8" s="20" t="s">
+      <c r="P8" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="O8" s="20" t="s">
+      <c r="Q8" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="P8" s="20" t="s">
+      <c r="R8" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="Q8" s="20" t="s">
+      <c r="S8" s="32" t="s">
         <v>32</v>
-      </c>
-      <c r="R8" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="S8" s="20" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:19">
-      <c r="B9" s="29"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="20"/>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="20"/>
-      <c r="R9" s="20"/>
-      <c r="S9" s="20"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="32"/>
+      <c r="Q9" s="32"/>
+      <c r="R9" s="32"/>
+      <c r="S9" s="32"/>
     </row>
     <row r="10" spans="2:19">
       <c r="B10" s="15"/>
@@ -1220,63 +1223,73 @@
       <c r="S10" s="18"/>
     </row>
     <row r="11" spans="2:19" ht="45">
-      <c r="B11" s="38">
+      <c r="B11" s="20">
         <v>1</v>
       </c>
       <c r="C11" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="F11" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="G11" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="H11" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="I11" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="J11" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="K11" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="19" t="s">
+      <c r="L11" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="K11" s="19" t="s">
+      <c r="M11" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="N11" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="M11" s="19" t="s">
+      <c r="O11" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="N11" s="19" t="s">
+      <c r="P11" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="O11" s="19" t="s">
+      <c r="Q11" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="R11" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="P11" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q11" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="R11" s="19" t="s">
-        <v>49</v>
-      </c>
       <c r="S11" s="19" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="H8:H9"/>
     <mergeCell ref="I8:I9"/>
@@ -1285,18 +1298,8 @@
     <mergeCell ref="Q8:Q9"/>
     <mergeCell ref="R8:R9"/>
     <mergeCell ref="S8:S9"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
     <mergeCell ref="O8:O9"/>
     <mergeCell ref="P8:P9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
   </mergeCells>
   <conditionalFormatting sqref="T2:T10">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Open">

</xml_diff>

<commit_message>
feat: implement auth controllers, add permission-based dashboard routing, and introduce template comparison utility
</commit_message>
<xml_diff>
--- a/public/tamplate-xlsx/Internal_Audit_Export_Tamplate.xlsx
+++ b/public/tamplate-xlsx/Internal_Audit_Export_Tamplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ict\www-wsl\qms\public\tamplate-xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EFB13E8-5AC0-401D-98A7-6587E5BE66AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6221F2D-BBEB-4DC2-B52C-C1242CE2FDA3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
   <si>
     <t xml:space="preserve">Rekap CAR Internal /Eksternal Audit </t>
   </si>
@@ -70,9 +70,6 @@
     <t>O</t>
   </si>
   <si>
-    <t>P</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -103,12 +100,6 @@
     <t>Findings</t>
   </si>
   <si>
-    <t>DEADLINE CAR SUBMIT</t>
-  </si>
-  <si>
-    <t>CAR STATUS</t>
-  </si>
-  <si>
     <t>Corrective Action</t>
   </si>
   <si>
@@ -155,9 +146,6 @@
   </si>
   <si>
     <t>16 Jul 2026</t>
-  </si>
-  <si>
-    <t>Under Review</t>
   </si>
   <si>
     <t>1. Corrective Action 1
@@ -174,13 +162,49 @@
   </si>
   <si>
     <t>Part No/Part Name/Process Checked</t>
+  </si>
+  <si>
+    <t>Nomor Dokumen</t>
+  </si>
+  <si>
+    <t>Departement</t>
+  </si>
+  <si>
+    <t>Tanggal Terbit</t>
+  </si>
+  <si>
+    <t>No Revisi</t>
+  </si>
+  <si>
+    <t>Halaman</t>
+  </si>
+  <si>
+    <t>: MANAGEMENT</t>
+  </si>
+  <si>
+    <t>: (Tanggal di Export)</t>
+  </si>
+  <si>
+    <t>: (Default 01)</t>
+  </si>
+  <si>
+    <t>: (Default 1 dari 1)</t>
+  </si>
+  <si>
+    <t>: (Tanggal di Export dan Angka Random di belakang)</t>
+  </si>
+  <si>
+    <t>Status Finding</t>
+  </si>
+  <si>
+    <t>Open</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -227,6 +251,11 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="DejaVu Sans"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -254,7 +283,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -353,41 +382,105 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -414,15 +507,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -441,89 +525,80 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF385724"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <b/>
@@ -964,11 +1039,13 @@
     <col min="5" max="5" width="14.7109375" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="10" max="11" width="12.5703125" customWidth="1"/>
-    <col min="13" max="13" width="36.5703125" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" customWidth="1"/>
-    <col min="16" max="16" width="28.85546875" customWidth="1"/>
-    <col min="17" max="17" width="12.7109375" customWidth="1"/>
-    <col min="18" max="18" width="28.85546875" customWidth="1"/>
+    <col min="12" max="12" width="12.140625" customWidth="1"/>
+    <col min="13" max="13" width="29.85546875" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" customWidth="1"/>
+    <col min="15" max="15" width="16.5703125" customWidth="1"/>
+    <col min="16" max="16" width="29.7109375" customWidth="1"/>
+    <col min="17" max="17" width="21.28515625" customWidth="1"/>
+    <col min="18" max="18" width="26.5703125" customWidth="1"/>
     <col min="19" max="19" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -976,105 +1053,125 @@
       <c r="B2" s="1"/>
       <c r="C2" s="2"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="24"/>
-      <c r="R2" s="24"/>
-      <c r="S2" s="25"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="31" t="s">
+        <v>46</v>
+      </c>
+      <c r="R2" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="S2" s="18"/>
     </row>
     <row r="3" spans="2:19" ht="15" customHeight="1">
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
-      <c r="N3" s="27"/>
-      <c r="O3" s="27"/>
-      <c r="P3" s="27"/>
-      <c r="Q3" s="27"/>
-      <c r="R3" s="27"/>
-      <c r="S3" s="28"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
+      <c r="N3" s="36"/>
+      <c r="O3" s="36"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="R3" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="S3" s="18"/>
     </row>
     <row r="4" spans="2:19" ht="15.75" customHeight="1">
       <c r="B4" s="4"/>
       <c r="C4" s="7"/>
       <c r="D4" s="8"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="28"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="37"/>
+      <c r="Q4" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="R4" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="S4" s="18"/>
     </row>
     <row r="5" spans="2:19" ht="15.75" customHeight="1">
       <c r="B5" s="4"/>
       <c r="C5" s="7"/>
       <c r="D5" s="8"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="28"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="36"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="R5" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="S5" s="18"/>
     </row>
     <row r="6" spans="2:19" ht="15" customHeight="1">
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="30"/>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="30"/>
-      <c r="O6" s="30"/>
-      <c r="P6" s="30"/>
-      <c r="Q6" s="30"/>
-      <c r="R6" s="30"/>
-      <c r="S6" s="31"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
+      <c r="L6" s="39"/>
+      <c r="M6" s="39"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="39"/>
+      <c r="P6" s="40"/>
+      <c r="Q6" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="R6" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="S6" s="18"/>
     </row>
     <row r="7" spans="2:19">
       <c r="B7" s="9"/>
@@ -1084,207 +1181,204 @@
       <c r="D7" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12" t="s">
+      <c r="G7" s="20"/>
+      <c r="H7" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="12" t="s">
+      <c r="J7" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="K7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="M7" s="12" t="s">
+      <c r="M7" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="N7" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="O7" s="12"/>
-      <c r="P7" s="13" t="s">
+      <c r="O7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="Q7" s="12" t="s">
+      <c r="P7" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="R7" s="12" t="s">
+      <c r="Q7" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="S7" s="14" t="s">
-        <v>16</v>
+      <c r="R7" s="20" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="2:19">
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="D8" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="E8" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="21" t="s">
+      <c r="G8" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="H8" s="21" t="s">
+      <c r="I8" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="J8" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="K8" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="K8" s="21" t="s">
+      <c r="L8" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="L8" s="21" t="s">
+      <c r="M8" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="M8" s="21" t="s">
+      <c r="N8" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="N8" s="32" t="s">
+      <c r="O8" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="O8" s="32" t="s">
+      <c r="P8" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="P8" s="32" t="s">
+      <c r="Q8" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="Q8" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="R8" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="S8" s="32" t="s">
-        <v>32</v>
+      <c r="R8" s="23" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="2:19">
-      <c r="B9" s="38"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="32"/>
-      <c r="O9" s="32"/>
-      <c r="P9" s="32"/>
-      <c r="Q9" s="32"/>
-      <c r="R9" s="32"/>
-      <c r="S9" s="32"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
+      <c r="Q9" s="23"/>
+      <c r="R9" s="23"/>
     </row>
     <row r="10" spans="2:19">
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="18"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
     </row>
     <row r="11" spans="2:19" ht="45">
-      <c r="B11" s="20">
+      <c r="B11" s="17">
         <v>1</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="G11" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="H11" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="I11" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="J11" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="K11" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="L11" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="J11" s="19" t="s">
+      <c r="M11" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="19" t="s">
+      <c r="N11" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="O11" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="L11" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="M11" s="19" t="s">
+      <c r="P11" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="N11" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="O11" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="P11" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q11" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="R11" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="S11" s="19" t="s">
-        <v>44</v>
+      <c r="Q11" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="R11" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="E2:P6"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="N8:N9"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
     <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D8:D9"/>
@@ -1293,39 +1387,17 @@
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="H8:H9"/>
     <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="E2:S6"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
   </mergeCells>
-  <conditionalFormatting sqref="T2:T10">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Open">
+  <conditionalFormatting sqref="T2:T6">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",T2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Closed">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Closed">
       <formula>NOT(ISERROR(SEARCH("Closed",T2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O11">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Open">
-      <formula>NOT(ISERROR(SEARCH("Open",O11)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="Closed">
-      <formula>NOT(ISERROR(SEARCH("Closed",O11)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T11">
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="Open">
-      <formula>NOT(ISERROR(SEARCH("Open",T11)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="Closed">
-      <formula>NOT(ISERROR(SEARCH("Closed",T11)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement DashboardController for audit data tracking and add internal audit export template
</commit_message>
<xml_diff>
--- a/public/tamplate-xlsx/Internal_Audit_Export_Tamplate.xlsx
+++ b/public/tamplate-xlsx/Internal_Audit_Export_Tamplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ict\www-wsl\qms\public\tamplate-xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6221F2D-BBEB-4DC2-B52C-C1242CE2FDA3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD2B363-8396-499D-998D-3552AB0EA1CD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -191,13 +191,13 @@
     <t>: (Default 1 dari 1)</t>
   </si>
   <si>
-    <t>: (Tanggal di Export dan Angka Random di belakang)</t>
-  </si>
-  <si>
     <t>Status Finding</t>
   </si>
   <si>
     <t>Open</t>
+  </si>
+  <si>
+    <t>: FO-08-02</t>
   </si>
 </sst>
 </file>
@@ -540,21 +540,51 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="15" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -563,66 +593,12 @@
     </xf>
     <xf numFmtId="15" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF385724"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <b/>
@@ -1053,25 +1029,25 @@
       <c r="B2" s="1"/>
       <c r="C2" s="2"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="32" t="s">
+      <c r="E2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="34"/>
-      <c r="Q2" s="31" t="s">
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="23" t="s">
         <v>46</v>
       </c>
       <c r="R2" s="22" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="S2" s="18"/>
     </row>
@@ -1079,19 +1055,19 @@
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="36"/>
-      <c r="P3" s="37"/>
-      <c r="Q3" s="31" t="s">
+      <c r="E3" s="30"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="23" t="s">
         <v>47</v>
       </c>
       <c r="R3" s="22" t="s">
@@ -1103,19 +1079,19 @@
       <c r="B4" s="4"/>
       <c r="C4" s="7"/>
       <c r="D4" s="8"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="37"/>
-      <c r="Q4" s="31" t="s">
+      <c r="E4" s="30"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="32"/>
+      <c r="Q4" s="23" t="s">
         <v>48</v>
       </c>
       <c r="R4" s="22" t="s">
@@ -1127,19 +1103,19 @@
       <c r="B5" s="4"/>
       <c r="C5" s="7"/>
       <c r="D5" s="8"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="31" t="s">
+      <c r="E5" s="30"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="32"/>
+      <c r="Q5" s="23" t="s">
         <v>49</v>
       </c>
       <c r="R5" s="22" t="s">
@@ -1148,24 +1124,24 @@
       <c r="S5" s="18"/>
     </row>
     <row r="6" spans="2:19" ht="15" customHeight="1">
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="39"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="39"/>
-      <c r="L6" s="39"/>
-      <c r="M6" s="39"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="39"/>
-      <c r="P6" s="40"/>
-      <c r="Q6" s="31" t="s">
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="34"/>
+      <c r="M6" s="34"/>
+      <c r="N6" s="34"/>
+      <c r="O6" s="34"/>
+      <c r="P6" s="35"/>
+      <c r="Q6" s="23" t="s">
         <v>50</v>
       </c>
       <c r="R6" s="22" t="s">
@@ -1223,76 +1199,76 @@
       </c>
     </row>
     <row r="8" spans="2:19">
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="H8" s="26" t="s">
+      <c r="H8" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="26" t="s">
+      <c r="I8" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="J8" s="26" t="s">
+      <c r="J8" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="K8" s="26" t="s">
+      <c r="K8" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="26" t="s">
+      <c r="L8" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="M8" s="26" t="s">
+      <c r="M8" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="N8" s="23" t="s">
+      <c r="N8" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="O8" s="23" t="s">
+      <c r="O8" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="P8" s="23" t="s">
+      <c r="P8" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="Q8" s="23" t="s">
+      <c r="Q8" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="R8" s="23" t="s">
-        <v>56</v>
+      <c r="R8" s="26" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="2:19">
-      <c r="B9" s="28"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
-      <c r="M9" s="27"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="23"/>
-      <c r="Q9" s="23"/>
-      <c r="R9" s="23"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="25"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="25"/>
+      <c r="M9" s="25"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="26"/>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="26"/>
+      <c r="R9" s="26"/>
     </row>
     <row r="10" spans="2:19">
       <c r="B10" s="12"/>
@@ -1363,18 +1339,11 @@
         <v>41</v>
       </c>
       <c r="R11" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="E2:P6"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="N8:N9"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
@@ -1387,12 +1356,19 @@
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="H8:H9"/>
     <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="E2:P6"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="N8:N9"/>
   </mergeCells>
   <conditionalFormatting sqref="T2:T6">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Open">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",T2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Closed">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Closed">
       <formula>NOT(ISERROR(SEARCH("Closed",T2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>